<commit_message>
Zinc Nuts and Smaller Washers
</commit_message>
<xml_diff>
--- a/resources/v0.1.1/design_documents/BOM-V0.1.1.xlsx
+++ b/resources/v0.1.1/design_documents/BOM-V0.1.1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\github\thermal-loop\resources\v0.1.1\design_documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/aimeehdz/Desktop/SMR Thermal Loop/thermal-loop/resources/v0.1.1/design_documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C9320B5-5B6A-4ECB-9EDA-3B007E86BC80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD2AFDC2-7D5C-8348-94E9-C88B8F040BE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FDAE7DA4-9528-4FC7-A320-70DA50473DCE}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" xr2:uid="{FDAE7DA4-9528-4FC7-A320-70DA50473DCE}"/>
   </bookViews>
   <sheets>
     <sheet name="bill_of_materials" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="402" uniqueCount="261">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="406" uniqueCount="263">
   <si>
     <t>Total Cost</t>
   </si>
@@ -819,6 +819,12 @@
   </si>
   <si>
     <t>Flange, 304 Stainless Steel, Metal Pipe Flange - 4WPV1 | Grainger</t>
+  </si>
+  <si>
+    <t>Zinc Coated</t>
+  </si>
+  <si>
+    <t>Need to be a smaller diameter</t>
   </si>
 </sst>
 </file>
@@ -908,7 +914,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -940,12 +946,21 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -982,10 +997,10 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1006,9 +1021,6 @@
     <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -1027,6 +1039,25 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1034,18 +1065,39 @@
   </cellStyles>
   <dxfs count="8">
     <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+      </border>
     </dxf>
     <dxf>
       <font>
@@ -1073,6 +1125,20 @@
         <family val="2"/>
         <scheme val="minor"/>
       </font>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0" outline="0">
         <left/>
@@ -1083,41 +1149,6 @@
         <bottom style="thin">
           <color theme="4" tint="0.39997558519241921"/>
         </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right/>
-        <top style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left/>
-        <right/>
-        <top style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
       </border>
     </dxf>
     <dxf>
@@ -1141,19 +1172,19 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{3AC99790-742C-414B-AF83-048E0365A8B5}" name="Table1" displayName="Table1" ref="A1:K103" totalsRowShown="0" tableBorderDxfId="7">
-  <autoFilter ref="A1:K103" xr:uid="{3AC99790-742C-414B-AF83-048E0365A8B5}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{3AC99790-742C-414B-AF83-048E0365A8B5}" name="Table1" displayName="Table1" ref="A1:K105" totalsRowShown="0" tableBorderDxfId="7">
+  <autoFilter ref="A1:K105" xr:uid="{3AC99790-742C-414B-AF83-048E0365A8B5}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{7B25C464-EB0A-4B56-94DE-96F6AA8DEAC1}" name="Internal Part Name" dataDxfId="2"/>
-    <tableColumn id="2" xr3:uid="{DF8C1AF7-50DF-4DF9-864F-041981FCACF8}" name="MFR / Vendor Description" dataDxfId="0"/>
-    <tableColumn id="3" xr3:uid="{352F414F-9DAD-4EB9-9018-5EFFD7851FC0}" name="MFR Part Number" dataDxfId="1"/>
-    <tableColumn id="4" xr3:uid="{524EB195-1154-4033-90BB-70DCBC8C6954}" name="Quantity" dataDxfId="4"/>
-    <tableColumn id="5" xr3:uid="{16A43733-D0E2-469A-A9F1-7003745CBA03}" name="Individual Cost" dataDxfId="6"/>
-    <tableColumn id="6" xr3:uid="{5E3D3D1D-3CF3-463A-8FD2-F7FCD175AFB0}" name="Total Cost" dataDxfId="5">
+    <tableColumn id="1" xr3:uid="{7B25C464-EB0A-4B56-94DE-96F6AA8DEAC1}" name="Internal Part Name" dataDxfId="6"/>
+    <tableColumn id="2" xr3:uid="{DF8C1AF7-50DF-4DF9-864F-041981FCACF8}" name="MFR / Vendor Description" dataDxfId="5"/>
+    <tableColumn id="3" xr3:uid="{352F414F-9DAD-4EB9-9018-5EFFD7851FC0}" name="MFR Part Number" dataDxfId="4"/>
+    <tableColumn id="4" xr3:uid="{524EB195-1154-4033-90BB-70DCBC8C6954}" name="Quantity" dataDxfId="3"/>
+    <tableColumn id="5" xr3:uid="{16A43733-D0E2-469A-A9F1-7003745CBA03}" name="Individual Cost" dataDxfId="2"/>
+    <tableColumn id="6" xr3:uid="{5E3D3D1D-3CF3-463A-8FD2-F7FCD175AFB0}" name="Total Cost" dataDxfId="1">
       <calculatedColumnFormula>D2*E2</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="7" xr3:uid="{75C60F91-0AB9-4643-82F8-4FD09187BCAB}" name="Notes"/>
-    <tableColumn id="8" xr3:uid="{B2E8A010-1D06-4803-ADB8-641F00C3F533}" name="Vendor 1" dataDxfId="3"/>
+    <tableColumn id="8" xr3:uid="{B2E8A010-1D06-4803-ADB8-641F00C3F533}" name="Vendor 1" dataDxfId="0"/>
     <tableColumn id="9" xr3:uid="{C1A08220-EBF0-49C3-9563-C3B6645758E0}" name="Vendor 2"/>
     <tableColumn id="10" xr3:uid="{D3EFF0C9-98BD-4B48-90E8-5030DBC5DB99}" name="Vendor 3"/>
     <tableColumn id="11" xr3:uid="{A06B68DA-A2F6-4D77-9FA7-22F7C10A75D6}" name="Vendor 4"/>
@@ -1480,24 +1511,24 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C6D3A36C-E8CE-4E50-A172-E48E2F9A45A8}">
   <dimension ref="A1:M109"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="20.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="33.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.42578125" customWidth="1"/>
+    <col min="1" max="1" width="20.1640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="33.1640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.83203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.5" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.5" customWidth="1"/>
     <col min="7" max="7" width="13" customWidth="1"/>
     <col min="8" max="8" width="79" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="45.5703125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="83.5703125" customWidth="1"/>
-    <col min="11" max="11" width="62.5703125" customWidth="1"/>
-    <col min="12" max="12" width="55.85546875" customWidth="1"/>
+    <col min="9" max="9" width="45.5" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="83.5" customWidth="1"/>
+    <col min="11" max="11" width="62.5" customWidth="1"/>
+    <col min="12" max="12" width="55.83203125" customWidth="1"/>
     <col min="13" max="13" width="51" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="8" t="s">
         <v>8</v>
       </c>
@@ -1532,11 +1563,11 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="28" t="s">
+      <c r="B2" s="27" t="s">
         <v>256</v>
       </c>
       <c r="C2" s="14">
@@ -1553,16 +1584,16 @@
         <v>25.58</v>
       </c>
       <c r="G2" s="5"/>
-      <c r="H2" s="24" t="s">
+      <c r="H2" s="23" t="s">
         <v>161</v>
       </c>
       <c r="J2" s="2"/>
     </row>
-    <row r="3" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="B3" s="28" t="s">
+      <c r="B3" s="27" t="s">
         <v>162</v>
       </c>
       <c r="C3" s="15">
@@ -1579,16 +1610,16 @@
         <v>17.100000000000001</v>
       </c>
       <c r="G3" s="5"/>
-      <c r="H3" s="25" t="s">
+      <c r="H3" s="24" t="s">
         <v>162</v>
       </c>
       <c r="I3" s="4"/>
     </row>
-    <row r="4" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="B4" s="28" t="s">
+      <c r="B4" s="27" t="s">
         <v>163</v>
       </c>
       <c r="C4" s="16">
@@ -1605,15 +1636,15 @@
         <v>4.6999999999999993</v>
       </c>
       <c r="G4" s="5"/>
-      <c r="H4" s="24" t="s">
+      <c r="H4" s="23" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="5" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="B5" s="28" t="s">
+      <c r="B5" s="27" t="s">
         <v>164</v>
       </c>
       <c r="C5" s="17">
@@ -1630,16 +1661,16 @@
         <v>32.700000000000003</v>
       </c>
       <c r="G5" s="5"/>
-      <c r="H5" s="25" t="s">
+      <c r="H5" s="24" t="s">
         <v>164</v>
       </c>
       <c r="I5" s="1"/>
     </row>
-    <row r="6" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="28" t="s">
+      <c r="B6" s="27" t="s">
         <v>165</v>
       </c>
       <c r="C6" s="18" t="s">
@@ -1656,16 +1687,16 @@
         <v>77.820000000000007</v>
       </c>
       <c r="G6" s="5"/>
-      <c r="H6" s="24" t="s">
+      <c r="H6" s="23" t="s">
         <v>165</v>
       </c>
       <c r="I6" s="4"/>
     </row>
-    <row r="7" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="B7" s="28" t="s">
+      <c r="B7" s="27" t="s">
         <v>166</v>
       </c>
       <c r="C7" s="19" t="s">
@@ -1682,18 +1713,18 @@
         <v>31.23</v>
       </c>
       <c r="G7" s="5"/>
-      <c r="H7" s="25" t="s">
+      <c r="H7" s="24" t="s">
         <v>166</v>
       </c>
       <c r="I7" s="4"/>
       <c r="J7" s="3"/>
       <c r="K7" s="3"/>
     </row>
-    <row r="8" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="28" t="s">
+      <c r="B8" s="27" t="s">
         <v>167</v>
       </c>
       <c r="C8" s="18" t="s">
@@ -1710,16 +1741,16 @@
         <v>93.93</v>
       </c>
       <c r="G8" s="5"/>
-      <c r="H8" s="24" t="s">
+      <c r="H8" s="23" t="s">
         <v>167</v>
       </c>
       <c r="I8" s="4"/>
     </row>
-    <row r="9" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="B9" s="28" t="s">
+      <c r="B9" s="27" t="s">
         <v>168</v>
       </c>
       <c r="C9" s="19" t="s">
@@ -1736,17 +1767,17 @@
         <v>5.99</v>
       </c>
       <c r="G9" s="5"/>
-      <c r="H9" s="25" t="s">
+      <c r="H9" s="24" t="s">
         <v>168</v>
       </c>
       <c r="L9" s="4"/>
       <c r="M9" s="4"/>
     </row>
-    <row r="10" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="B10" s="28" t="s">
+      <c r="B10" s="27" t="s">
         <v>169</v>
       </c>
       <c r="C10" s="18" t="s">
@@ -1763,15 +1794,15 @@
         <v>41.22</v>
       </c>
       <c r="G10" s="5"/>
-      <c r="H10" s="24" t="s">
+      <c r="H10" s="23" t="s">
         <v>169</v>
       </c>
     </row>
-    <row r="11" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="B11" s="28" t="s">
+      <c r="B11" s="27" t="s">
         <v>170</v>
       </c>
       <c r="C11" s="19" t="s">
@@ -1788,16 +1819,16 @@
         <v>60.89</v>
       </c>
       <c r="G11" s="5"/>
-      <c r="H11" s="25" t="s">
+      <c r="H11" s="24" t="s">
         <v>170</v>
       </c>
       <c r="I11" s="3"/>
     </row>
-    <row r="12" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="14" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="28"/>
+      <c r="B12" s="27"/>
       <c r="C12" s="14" t="s">
         <v>81</v>
       </c>
@@ -1812,16 +1843,16 @@
         <v>27.83</v>
       </c>
       <c r="G12" s="5"/>
-      <c r="H12" s="26" t="s">
+      <c r="H12" s="25" t="s">
         <v>81</v>
       </c>
       <c r="I12" s="4"/>
     </row>
-    <row r="13" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="B13" s="28" t="s">
+      <c r="B13" s="27" t="s">
         <v>171</v>
       </c>
       <c r="C13" s="20">
@@ -1838,16 +1869,16 @@
         <v>370</v>
       </c>
       <c r="G13" s="5"/>
-      <c r="H13" s="25" t="s">
+      <c r="H13" s="24" t="s">
         <v>171</v>
       </c>
       <c r="I13" s="4"/>
     </row>
-    <row r="14" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="14" t="s">
         <v>20</v>
       </c>
-      <c r="B14" s="28" t="s">
+      <c r="B14" s="27" t="s">
         <v>172</v>
       </c>
       <c r="C14" s="18">
@@ -1864,16 +1895,16 @@
         <v>312</v>
       </c>
       <c r="G14" s="5"/>
-      <c r="H14" s="24" t="s">
+      <c r="H14" s="23" t="s">
         <v>172</v>
       </c>
       <c r="I14" s="4"/>
     </row>
-    <row r="15" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="B15" s="28" t="s">
+      <c r="B15" s="27" t="s">
         <v>173</v>
       </c>
       <c r="C15" s="20">
@@ -1890,16 +1921,16 @@
         <v>5.9</v>
       </c>
       <c r="G15" s="5"/>
-      <c r="H15" s="25" t="s">
+      <c r="H15" s="24" t="s">
         <v>173</v>
       </c>
       <c r="I15" s="4"/>
     </row>
-    <row r="16" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="B16" s="28" t="s">
+      <c r="B16" s="27" t="s">
         <v>174</v>
       </c>
       <c r="C16" s="21">
@@ -1916,16 +1947,16 @@
         <v>1610</v>
       </c>
       <c r="G16" s="5"/>
-      <c r="H16" s="24" t="s">
+      <c r="H16" s="23" t="s">
         <v>174</v>
       </c>
       <c r="I16" s="4"/>
     </row>
-    <row r="17" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="B17" s="28" t="s">
+      <c r="B17" s="27" t="s">
         <v>175</v>
       </c>
       <c r="C17" s="15" t="s">
@@ -1942,16 +1973,16 @@
         <v>99.25</v>
       </c>
       <c r="G17" s="5"/>
-      <c r="H17" s="25" t="s">
+      <c r="H17" s="24" t="s">
         <v>175</v>
       </c>
       <c r="I17" s="4"/>
     </row>
-    <row r="18" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="14" t="s">
         <v>24</v>
       </c>
-      <c r="B18" s="28"/>
+      <c r="B18" s="27"/>
       <c r="C18" s="14" t="s">
         <v>83</v>
       </c>
@@ -1966,16 +1997,16 @@
         <v>839.97</v>
       </c>
       <c r="G18" s="5"/>
-      <c r="H18" s="26" t="s">
+      <c r="H18" s="25" t="s">
         <v>81</v>
       </c>
       <c r="I18" s="4"/>
     </row>
-    <row r="19" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="B19" s="28" t="s">
+      <c r="B19" s="27" t="s">
         <v>176</v>
       </c>
       <c r="C19" s="15" t="s">
@@ -1992,16 +2023,16 @@
         <v>28.04</v>
       </c>
       <c r="G19" s="5"/>
-      <c r="H19" s="25" t="s">
+      <c r="H19" s="24" t="s">
         <v>176</v>
       </c>
       <c r="I19" s="4"/>
     </row>
-    <row r="20" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="B20" s="28" t="s">
+      <c r="B20" s="27" t="s">
         <v>177</v>
       </c>
       <c r="C20" s="14" t="s">
@@ -2018,16 +2049,16 @@
         <v>33.58</v>
       </c>
       <c r="G20" s="5"/>
-      <c r="H20" s="24" t="s">
+      <c r="H20" s="23" t="s">
         <v>177</v>
       </c>
       <c r="I20" s="4"/>
     </row>
-    <row r="21" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="B21" s="28" t="s">
+      <c r="B21" s="27" t="s">
         <v>178</v>
       </c>
       <c r="C21" s="15" t="s">
@@ -2044,16 +2075,16 @@
         <v>31.66</v>
       </c>
       <c r="G21" s="5"/>
-      <c r="H21" s="25" t="s">
+      <c r="H21" s="24" t="s">
         <v>178</v>
       </c>
       <c r="I21" s="4"/>
     </row>
-    <row r="22" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="B22" s="28" t="s">
+      <c r="B22" s="27" t="s">
         <v>179</v>
       </c>
       <c r="C22" s="14" t="s">
@@ -2070,16 +2101,16 @@
         <v>59</v>
       </c>
       <c r="G22" s="5"/>
-      <c r="H22" s="24" t="s">
+      <c r="H22" s="23" t="s">
         <v>179</v>
       </c>
       <c r="I22" s="4"/>
     </row>
-    <row r="23" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="15" t="s">
         <v>29</v>
       </c>
-      <c r="B23" s="28" t="s">
+      <c r="B23" s="27" t="s">
         <v>180</v>
       </c>
       <c r="C23" s="15">
@@ -2096,16 +2127,16 @@
         <v>682.26</v>
       </c>
       <c r="G23" s="5"/>
-      <c r="H23" s="25" t="s">
+      <c r="H23" s="24" t="s">
         <v>180</v>
       </c>
       <c r="I23" s="4"/>
     </row>
-    <row r="24" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="14" t="s">
         <v>30</v>
       </c>
-      <c r="B24" s="28" t="s">
+      <c r="B24" s="27" t="s">
         <v>181</v>
       </c>
       <c r="C24" s="14">
@@ -2122,16 +2153,16 @@
         <v>216.04</v>
       </c>
       <c r="G24" s="5"/>
-      <c r="H24" s="24" t="s">
+      <c r="H24" s="23" t="s">
         <v>181</v>
       </c>
       <c r="I24" s="4"/>
     </row>
-    <row r="25" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="B25" s="28" t="s">
+      <c r="B25" s="27" t="s">
         <v>179</v>
       </c>
       <c r="C25" s="15" t="s">
@@ -2148,16 +2179,16 @@
         <v>295</v>
       </c>
       <c r="G25" s="2"/>
-      <c r="H25" s="25" t="s">
+      <c r="H25" s="24" t="s">
         <v>179</v>
       </c>
       <c r="I25" s="4"/>
     </row>
-    <row r="26" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="14" t="s">
         <v>31</v>
       </c>
-      <c r="B26" s="28" t="s">
+      <c r="B26" s="27" t="s">
         <v>182</v>
       </c>
       <c r="C26" s="14" t="s">
@@ -2174,16 +2205,16 @@
         <v>83.96</v>
       </c>
       <c r="G26" s="2"/>
-      <c r="H26" s="24" t="s">
+      <c r="H26" s="23" t="s">
         <v>182</v>
       </c>
       <c r="I26" s="2"/>
     </row>
-    <row r="27" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="B27" s="28" t="s">
+      <c r="B27" s="27" t="s">
         <v>183</v>
       </c>
       <c r="C27" s="19" t="s">
@@ -2200,15 +2231,15 @@
         <v>29.84</v>
       </c>
       <c r="G27" s="2"/>
-      <c r="H27" s="25" t="s">
+      <c r="H27" s="24" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="28" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="B28" s="28" t="s">
+      <c r="B28" s="27" t="s">
         <v>184</v>
       </c>
       <c r="C28" s="18" t="s">
@@ -2224,15 +2255,15 @@
         <f t="shared" si="0"/>
         <v>52.92</v>
       </c>
-      <c r="H28" s="24" t="s">
+      <c r="H28" s="23" t="s">
         <v>184</v>
       </c>
     </row>
-    <row r="29" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="15" t="s">
         <v>33</v>
       </c>
-      <c r="B29" s="28" t="s">
+      <c r="B29" s="27" t="s">
         <v>185</v>
       </c>
       <c r="C29" s="15" t="s">
@@ -2248,15 +2279,15 @@
         <f t="shared" si="0"/>
         <v>51.12</v>
       </c>
-      <c r="H29" s="25" t="s">
+      <c r="H29" s="24" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="30" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="14" t="s">
         <v>34</v>
       </c>
-      <c r="B30" s="28" t="s">
+      <c r="B30" s="27" t="s">
         <v>186</v>
       </c>
       <c r="C30" s="18" t="s">
@@ -2272,15 +2303,15 @@
         <f t="shared" si="0"/>
         <v>39.96</v>
       </c>
-      <c r="H30" s="24" t="s">
+      <c r="H30" s="23" t="s">
         <v>186</v>
       </c>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A31" s="15" t="s">
         <v>35</v>
       </c>
-      <c r="B31" s="28" t="s">
+      <c r="B31" s="27" t="s">
         <v>187</v>
       </c>
       <c r="C31" s="19" t="s">
@@ -2296,15 +2327,15 @@
         <f t="shared" si="0"/>
         <v>89.36</v>
       </c>
-      <c r="H31" s="25" t="s">
+      <c r="H31" s="24" t="s">
         <v>187</v>
       </c>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A32" s="14" t="s">
         <v>35</v>
       </c>
-      <c r="B32" s="28" t="s">
+      <c r="B32" s="27" t="s">
         <v>188</v>
       </c>
       <c r="C32" s="18" t="s">
@@ -2320,15 +2351,15 @@
         <f t="shared" si="0"/>
         <v>67.56</v>
       </c>
-      <c r="H32" s="24" t="s">
+      <c r="H32" s="23" t="s">
         <v>188</v>
       </c>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A33" s="15" t="s">
         <v>36</v>
       </c>
-      <c r="B33" s="28" t="s">
+      <c r="B33" s="27" t="s">
         <v>189</v>
       </c>
       <c r="C33" s="19" t="s">
@@ -2344,15 +2375,15 @@
         <f t="shared" si="0"/>
         <v>43.58</v>
       </c>
-      <c r="H33" s="25" t="s">
+      <c r="H33" s="24" t="s">
         <v>189</v>
       </c>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A34" s="14" t="s">
         <v>36</v>
       </c>
-      <c r="B34" s="28" t="s">
+      <c r="B34" s="27" t="s">
         <v>190</v>
       </c>
       <c r="C34" s="18" t="s">
@@ -2368,15 +2399,15 @@
         <f t="shared" si="0"/>
         <v>39.72</v>
       </c>
-      <c r="H34" s="24" t="s">
+      <c r="H34" s="23" t="s">
         <v>190</v>
       </c>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A35" s="15" t="s">
         <v>37</v>
       </c>
-      <c r="B35" s="28" t="s">
+      <c r="B35" s="27" t="s">
         <v>191</v>
       </c>
       <c r="C35" s="19" t="s">
@@ -2392,15 +2423,15 @@
         <f t="shared" si="0"/>
         <v>36.979999999999997</v>
       </c>
-      <c r="H35" s="25" t="s">
+      <c r="H35" s="24" t="s">
         <v>191</v>
       </c>
     </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A36" s="14" t="s">
         <v>37</v>
       </c>
-      <c r="B36" s="28" t="s">
+      <c r="B36" s="27" t="s">
         <v>192</v>
       </c>
       <c r="C36" s="18" t="s">
@@ -2416,15 +2447,15 @@
         <f t="shared" si="0"/>
         <v>26.2</v>
       </c>
-      <c r="H36" s="24" t="s">
+      <c r="H36" s="23" t="s">
         <v>192</v>
       </c>
     </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A37" s="15" t="s">
         <v>35</v>
       </c>
-      <c r="B37" s="28" t="s">
+      <c r="B37" s="27" t="s">
         <v>193</v>
       </c>
       <c r="C37" s="19" t="s">
@@ -2440,15 +2471,15 @@
         <f t="shared" si="0"/>
         <v>76.88</v>
       </c>
-      <c r="H37" s="25" t="s">
+      <c r="H37" s="24" t="s">
         <v>193</v>
       </c>
     </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A38" s="14" t="s">
         <v>38</v>
       </c>
-      <c r="B38" s="28" t="s">
+      <c r="B38" s="27" t="s">
         <v>194</v>
       </c>
       <c r="C38" s="18" t="s">
@@ -2464,15 +2495,15 @@
         <f t="shared" si="0"/>
         <v>14.879999999999999</v>
       </c>
-      <c r="H38" s="24" t="s">
+      <c r="H38" s="23" t="s">
         <v>194</v>
       </c>
     </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A39" s="15" t="s">
         <v>38</v>
       </c>
-      <c r="B39" s="28" t="s">
+      <c r="B39" s="27" t="s">
         <v>195</v>
       </c>
       <c r="C39" s="19" t="s">
@@ -2488,15 +2519,15 @@
         <f t="shared" si="0"/>
         <v>19.259999999999998</v>
       </c>
-      <c r="H39" s="25" t="s">
+      <c r="H39" s="24" t="s">
         <v>195</v>
       </c>
     </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A40" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="B40" s="28" t="s">
+      <c r="B40" s="27" t="s">
         <v>196</v>
       </c>
       <c r="C40" s="18" t="s">
@@ -2512,15 +2543,15 @@
         <f t="shared" si="0"/>
         <v>16.010000000000002</v>
       </c>
-      <c r="H40" s="24" t="s">
+      <c r="H40" s="23" t="s">
         <v>196</v>
       </c>
     </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A41" s="15" t="s">
         <v>39</v>
       </c>
-      <c r="B41" s="28" t="s">
+      <c r="B41" s="27" t="s">
         <v>257</v>
       </c>
       <c r="C41" s="19" t="s">
@@ -2536,15 +2567,15 @@
         <f t="shared" si="0"/>
         <v>22.65</v>
       </c>
-      <c r="H41" s="25" t="s">
+      <c r="H41" s="24" t="s">
         <v>197</v>
       </c>
     </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A42" s="14" t="s">
         <v>40</v>
       </c>
-      <c r="B42" s="28" t="s">
+      <c r="B42" s="27" t="s">
         <v>198</v>
       </c>
       <c r="C42" s="18" t="s">
@@ -2560,15 +2591,15 @@
         <f t="shared" si="0"/>
         <v>42.599999999999994</v>
       </c>
-      <c r="H42" s="24" t="s">
+      <c r="H42" s="23" t="s">
         <v>198</v>
       </c>
     </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A43" s="15" t="s">
         <v>41</v>
       </c>
-      <c r="B43" s="28" t="s">
+      <c r="B43" s="27" t="s">
         <v>199</v>
       </c>
       <c r="C43" s="19" t="s">
@@ -2584,15 +2615,15 @@
         <f t="shared" si="0"/>
         <v>50.51</v>
       </c>
-      <c r="H43" s="25" t="s">
+      <c r="H43" s="24" t="s">
         <v>199</v>
       </c>
     </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A44" s="14" t="s">
         <v>42</v>
       </c>
-      <c r="B44" s="28" t="s">
+      <c r="B44" s="27" t="s">
         <v>200</v>
       </c>
       <c r="C44" s="18" t="s">
@@ -2608,15 +2639,15 @@
         <f t="shared" si="0"/>
         <v>24.17</v>
       </c>
-      <c r="H44" s="24" t="s">
+      <c r="H44" s="23" t="s">
         <v>200</v>
       </c>
     </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A45" s="15" t="s">
         <v>43</v>
       </c>
-      <c r="B45" s="28" t="s">
+      <c r="B45" s="27" t="s">
         <v>201</v>
       </c>
       <c r="C45" s="19" t="s">
@@ -2632,15 +2663,15 @@
         <f t="shared" si="0"/>
         <v>26.01</v>
       </c>
-      <c r="H45" s="25" t="s">
+      <c r="H45" s="24" t="s">
         <v>201</v>
       </c>
     </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A46" s="14" t="s">
         <v>44</v>
       </c>
-      <c r="B46" s="28" t="s">
+      <c r="B46" s="27" t="s">
         <v>202</v>
       </c>
       <c r="C46" s="18" t="s">
@@ -2656,15 +2687,15 @@
         <f t="shared" si="0"/>
         <v>16.82</v>
       </c>
-      <c r="H46" s="24" t="s">
+      <c r="H46" s="23" t="s">
         <v>202</v>
       </c>
     </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A47" s="15" t="s">
         <v>45</v>
       </c>
-      <c r="B47" s="28" t="s">
+      <c r="B47" s="27" t="s">
         <v>203</v>
       </c>
       <c r="C47" s="19" t="s">
@@ -2680,15 +2711,15 @@
         <f t="shared" si="0"/>
         <v>50.34</v>
       </c>
-      <c r="H47" s="25" t="s">
+      <c r="H47" s="24" t="s">
         <v>203</v>
       </c>
     </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A48" s="14" t="s">
         <v>45</v>
       </c>
-      <c r="B48" s="28" t="s">
+      <c r="B48" s="27" t="s">
         <v>204</v>
       </c>
       <c r="C48" s="18" t="s">
@@ -2704,15 +2735,15 @@
         <f t="shared" si="0"/>
         <v>25</v>
       </c>
-      <c r="H48" s="24" t="s">
+      <c r="H48" s="23" t="s">
         <v>204</v>
       </c>
     </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A49" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="B49" s="28" t="s">
+      <c r="B49" s="27" t="s">
         <v>205</v>
       </c>
       <c r="C49" s="19" t="s">
@@ -2728,15 +2759,15 @@
         <f t="shared" si="0"/>
         <v>28.56</v>
       </c>
-      <c r="H49" s="25" t="s">
+      <c r="H49" s="24" t="s">
         <v>205</v>
       </c>
     </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A50" s="14" t="s">
         <v>47</v>
       </c>
-      <c r="B50" s="28" t="s">
+      <c r="B50" s="27" t="s">
         <v>206</v>
       </c>
       <c r="C50" s="18" t="s">
@@ -2752,15 +2783,15 @@
         <f t="shared" si="0"/>
         <v>16.75</v>
       </c>
-      <c r="H50" s="24" t="s">
+      <c r="H50" s="23" t="s">
         <v>206</v>
       </c>
     </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A51" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="B51" s="28" t="s">
+      <c r="B51" s="27" t="s">
         <v>207</v>
       </c>
       <c r="C51" s="19" t="s">
@@ -2776,15 +2807,15 @@
         <f t="shared" si="0"/>
         <v>14.81</v>
       </c>
-      <c r="H51" s="25" t="s">
+      <c r="H51" s="24" t="s">
         <v>207</v>
       </c>
     </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A52" s="14" t="s">
         <v>46</v>
       </c>
-      <c r="B52" s="28" t="s">
+      <c r="B52" s="27" t="s">
         <v>208</v>
       </c>
       <c r="C52" s="18" t="s">
@@ -2800,15 +2831,15 @@
         <f t="shared" si="0"/>
         <v>19.989999999999998</v>
       </c>
-      <c r="H52" s="24" t="s">
+      <c r="H52" s="23" t="s">
         <v>208</v>
       </c>
     </row>
-    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A53" s="15" t="s">
         <v>48</v>
       </c>
-      <c r="B53" s="28" t="s">
+      <c r="B53" s="27" t="s">
         <v>209</v>
       </c>
       <c r="C53" s="19" t="s">
@@ -2824,15 +2855,15 @@
         <f t="shared" si="0"/>
         <v>26.8</v>
       </c>
-      <c r="H53" s="25" t="s">
+      <c r="H53" s="24" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A54" s="14" t="s">
         <v>49</v>
       </c>
-      <c r="B54" s="28" t="s">
+      <c r="B54" s="27" t="s">
         <v>210</v>
       </c>
       <c r="C54" s="18" t="s">
@@ -2848,15 +2879,15 @@
         <f t="shared" si="0"/>
         <v>40.14</v>
       </c>
-      <c r="H54" s="24" t="s">
+      <c r="H54" s="23" t="s">
         <v>210</v>
       </c>
     </row>
-    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A55" s="15" t="s">
         <v>50</v>
       </c>
-      <c r="B55" s="28" t="s">
+      <c r="B55" s="27" t="s">
         <v>211</v>
       </c>
       <c r="C55" s="15" t="s">
@@ -2872,15 +2903,15 @@
         <f t="shared" si="0"/>
         <v>300</v>
       </c>
-      <c r="H55" s="25" t="s">
+      <c r="H55" s="24" t="s">
         <v>211</v>
       </c>
     </row>
-    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A56" s="14" t="s">
         <v>35</v>
       </c>
-      <c r="B56" s="28" t="s">
+      <c r="B56" s="27" t="s">
         <v>212</v>
       </c>
       <c r="C56" s="18" t="s">
@@ -2896,15 +2927,15 @@
         <f t="shared" si="0"/>
         <v>69.179999999999993</v>
       </c>
-      <c r="H56" s="24" t="s">
+      <c r="H56" s="23" t="s">
         <v>212</v>
       </c>
     </row>
-    <row r="57" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A57" s="15" t="s">
         <v>48</v>
       </c>
-      <c r="B57" s="28" t="s">
+      <c r="B57" s="27" t="s">
         <v>213</v>
       </c>
       <c r="C57" s="19" t="s">
@@ -2920,15 +2951,15 @@
         <f t="shared" si="0"/>
         <v>9.5</v>
       </c>
-      <c r="H57" s="25" t="s">
+      <c r="H57" s="24" t="s">
         <v>213</v>
       </c>
     </row>
-    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A58" s="14" t="s">
         <v>39</v>
       </c>
-      <c r="B58" s="28" t="s">
+      <c r="B58" s="27" t="s">
         <v>214</v>
       </c>
       <c r="C58" s="18" t="s">
@@ -2944,15 +2975,15 @@
         <f t="shared" si="0"/>
         <v>5.41</v>
       </c>
-      <c r="H58" s="24" t="s">
+      <c r="H58" s="23" t="s">
         <v>214</v>
       </c>
     </row>
-    <row r="59" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A59" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="B59" s="28" t="s">
+      <c r="B59" s="27" t="s">
         <v>215</v>
       </c>
       <c r="C59" s="19" t="s">
@@ -2968,15 +2999,15 @@
         <f t="shared" si="0"/>
         <v>9.0299999999999994</v>
       </c>
-      <c r="H59" s="25" t="s">
+      <c r="H59" s="24" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A60" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="B60" s="28" t="s">
+      <c r="B60" s="27" t="s">
         <v>216</v>
       </c>
       <c r="C60" s="18" t="s">
@@ -2992,15 +3023,15 @@
         <f t="shared" si="0"/>
         <v>16.87</v>
       </c>
-      <c r="H60" s="24" t="s">
+      <c r="H60" s="23" t="s">
         <v>216</v>
       </c>
     </row>
-    <row r="61" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A61" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="B61" s="28" t="s">
+      <c r="B61" s="27" t="s">
         <v>217</v>
       </c>
       <c r="C61" s="19" t="s">
@@ -3016,15 +3047,15 @@
         <f t="shared" si="0"/>
         <v>14.02</v>
       </c>
-      <c r="H61" s="25" t="s">
+      <c r="H61" s="24" t="s">
         <v>217</v>
       </c>
     </row>
-    <row r="62" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A62" s="14" t="s">
         <v>52</v>
       </c>
-      <c r="B62" s="28" t="s">
+      <c r="B62" s="27" t="s">
         <v>218</v>
       </c>
       <c r="C62" s="18" t="s">
@@ -3040,15 +3071,15 @@
         <f t="shared" si="0"/>
         <v>8.83</v>
       </c>
-      <c r="H62" s="24" t="s">
+      <c r="H62" s="23" t="s">
         <v>218</v>
       </c>
     </row>
-    <row r="63" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A63" s="15" t="s">
         <v>52</v>
       </c>
-      <c r="B63" s="28" t="s">
+      <c r="B63" s="27" t="s">
         <v>219</v>
       </c>
       <c r="C63" s="19" t="s">
@@ -3064,15 +3095,15 @@
         <f t="shared" si="0"/>
         <v>7.19</v>
       </c>
-      <c r="H63" s="25" t="s">
+      <c r="H63" s="24" t="s">
         <v>219</v>
       </c>
     </row>
-    <row r="64" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A64" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B64" s="28" t="s">
+      <c r="B64" s="27" t="s">
         <v>220</v>
       </c>
       <c r="C64" s="18" t="s">
@@ -3088,15 +3119,15 @@
         <f t="shared" si="0"/>
         <v>11.04</v>
       </c>
-      <c r="H64" s="24" t="s">
+      <c r="H64" s="23" t="s">
         <v>220</v>
       </c>
     </row>
-    <row r="65" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A65" s="15" t="s">
         <v>45</v>
       </c>
-      <c r="B65" s="28" t="s">
+      <c r="B65" s="27" t="s">
         <v>221</v>
       </c>
       <c r="C65" s="19" t="s">
@@ -3112,15 +3143,15 @@
         <f t="shared" si="0"/>
         <v>6.98</v>
       </c>
-      <c r="H65" s="25" t="s">
+      <c r="H65" s="24" t="s">
         <v>221</v>
       </c>
     </row>
-    <row r="66" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A66" s="14" t="s">
         <v>37</v>
       </c>
-      <c r="B66" s="28" t="s">
+      <c r="B66" s="27" t="s">
         <v>222</v>
       </c>
       <c r="C66" s="18" t="s">
@@ -3136,15 +3167,15 @@
         <f t="shared" si="0"/>
         <v>42.76</v>
       </c>
-      <c r="H66" s="24" t="s">
+      <c r="H66" s="23" t="s">
         <v>222</v>
       </c>
     </row>
-    <row r="67" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A67" s="15" t="s">
         <v>53</v>
       </c>
-      <c r="B67" s="28" t="s">
+      <c r="B67" s="27" t="s">
         <v>223</v>
       </c>
       <c r="C67" s="19" t="s">
@@ -3160,15 +3191,15 @@
         <f t="shared" ref="F67:F103" si="1">D67*E67</f>
         <v>45.81</v>
       </c>
-      <c r="H67" s="25" t="s">
+      <c r="H67" s="24" t="s">
         <v>223</v>
       </c>
     </row>
-    <row r="68" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A68" s="14" t="s">
         <v>45</v>
       </c>
-      <c r="B68" s="28" t="s">
+      <c r="B68" s="27" t="s">
         <v>224</v>
       </c>
       <c r="C68" s="18" t="s">
@@ -3184,15 +3215,15 @@
         <f t="shared" si="1"/>
         <v>18.73</v>
       </c>
-      <c r="H68" s="24" t="s">
+      <c r="H68" s="23" t="s">
         <v>224</v>
       </c>
     </row>
-    <row r="69" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A69" s="15" t="s">
         <v>54</v>
       </c>
-      <c r="B69" s="28" t="s">
+      <c r="B69" s="27" t="s">
         <v>225</v>
       </c>
       <c r="C69" s="19" t="s">
@@ -3208,15 +3239,15 @@
         <f t="shared" si="1"/>
         <v>4.99</v>
       </c>
-      <c r="H69" s="25" t="s">
+      <c r="H69" s="24" t="s">
         <v>225</v>
       </c>
     </row>
-    <row r="70" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A70" s="14" t="s">
         <v>54</v>
       </c>
-      <c r="B70" s="28" t="s">
+      <c r="B70" s="27" t="s">
         <v>226</v>
       </c>
       <c r="C70" s="18" t="s">
@@ -3232,15 +3263,15 @@
         <f t="shared" si="1"/>
         <v>4.68</v>
       </c>
-      <c r="H70" s="24" t="s">
+      <c r="H70" s="23" t="s">
         <v>226</v>
       </c>
     </row>
-    <row r="71" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A71" s="15" t="s">
         <v>55</v>
       </c>
-      <c r="B71" s="28" t="s">
+      <c r="B71" s="27" t="s">
         <v>227</v>
       </c>
       <c r="C71" s="19" t="s">
@@ -3256,15 +3287,15 @@
         <f t="shared" si="1"/>
         <v>39.72</v>
       </c>
-      <c r="H71" s="25" t="s">
+      <c r="H71" s="24" t="s">
         <v>227</v>
       </c>
     </row>
-    <row r="72" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A72" s="14" t="s">
         <v>46</v>
       </c>
-      <c r="B72" s="28" t="s">
+      <c r="B72" s="27" t="s">
         <v>228</v>
       </c>
       <c r="C72" s="18" t="s">
@@ -3280,15 +3311,15 @@
         <f t="shared" si="1"/>
         <v>15.07</v>
       </c>
-      <c r="H72" s="24" t="s">
+      <c r="H72" s="23" t="s">
         <v>228</v>
       </c>
     </row>
-    <row r="73" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A73" s="15" t="s">
         <v>56</v>
       </c>
-      <c r="B73" s="28" t="s">
+      <c r="B73" s="27" t="s">
         <v>229</v>
       </c>
       <c r="C73" s="19" t="s">
@@ -3304,15 +3335,15 @@
         <f t="shared" si="1"/>
         <v>45.58</v>
       </c>
-      <c r="H73" s="25" t="s">
+      <c r="H73" s="24" t="s">
         <v>229</v>
       </c>
     </row>
-    <row r="74" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A74" s="14" t="s">
         <v>57</v>
       </c>
-      <c r="B74" s="28" t="s">
+      <c r="B74" s="27" t="s">
         <v>230</v>
       </c>
       <c r="C74" s="18" t="s">
@@ -3328,15 +3359,15 @@
         <f t="shared" si="1"/>
         <v>6.43</v>
       </c>
-      <c r="H74" s="24" t="s">
+      <c r="H74" s="23" t="s">
         <v>230</v>
       </c>
     </row>
-    <row r="75" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A75" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="B75" s="28" t="s">
+      <c r="B75" s="27" t="s">
         <v>231</v>
       </c>
       <c r="C75" s="19" t="s">
@@ -3352,15 +3383,15 @@
         <f t="shared" si="1"/>
         <v>26.5</v>
       </c>
-      <c r="H75" s="25" t="s">
+      <c r="H75" s="24" t="s">
         <v>231</v>
       </c>
     </row>
-    <row r="76" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A76" s="14" t="s">
         <v>58</v>
       </c>
-      <c r="B76" s="28" t="s">
+      <c r="B76" s="27" t="s">
         <v>232</v>
       </c>
       <c r="C76" s="14" t="s">
@@ -3376,15 +3407,15 @@
         <f t="shared" si="1"/>
         <v>25.6</v>
       </c>
-      <c r="H76" s="24" t="s">
+      <c r="H76" s="23" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="77" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A77" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="B77" s="28" t="s">
+      <c r="B77" s="27" t="s">
         <v>233</v>
       </c>
       <c r="C77" s="19" t="s">
@@ -3400,15 +3431,15 @@
         <f t="shared" si="1"/>
         <v>14.16</v>
       </c>
-      <c r="H77" s="25" t="s">
+      <c r="H77" s="24" t="s">
         <v>233</v>
       </c>
     </row>
-    <row r="78" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A78" s="14" t="s">
         <v>39</v>
       </c>
-      <c r="B78" s="28" t="s">
+      <c r="B78" s="27" t="s">
         <v>234</v>
       </c>
       <c r="C78" s="18" t="s">
@@ -3424,15 +3455,15 @@
         <f t="shared" si="1"/>
         <v>34.900000000000006</v>
       </c>
-      <c r="H78" s="24" t="s">
+      <c r="H78" s="23" t="s">
         <v>234</v>
       </c>
     </row>
-    <row r="79" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A79" s="15" t="s">
         <v>59</v>
       </c>
-      <c r="B79" s="28" t="s">
+      <c r="B79" s="27" t="s">
         <v>235</v>
       </c>
       <c r="C79" s="19" t="s">
@@ -3448,15 +3479,15 @@
         <f t="shared" si="1"/>
         <v>3.76</v>
       </c>
-      <c r="H79" s="25" t="s">
+      <c r="H79" s="24" t="s">
         <v>235</v>
       </c>
     </row>
-    <row r="80" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A80" s="14" t="s">
         <v>60</v>
       </c>
-      <c r="B80" s="28" t="s">
+      <c r="B80" s="27" t="s">
         <v>236</v>
       </c>
       <c r="C80" s="18" t="s">
@@ -3472,15 +3503,15 @@
         <f t="shared" si="1"/>
         <v>4.72</v>
       </c>
-      <c r="H80" s="24" t="s">
+      <c r="H80" s="23" t="s">
         <v>236</v>
       </c>
     </row>
-    <row r="81" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A81" s="15" t="s">
         <v>61</v>
       </c>
-      <c r="B81" s="28" t="s">
+      <c r="B81" s="27" t="s">
         <v>237</v>
       </c>
       <c r="C81" s="19" t="s">
@@ -3496,15 +3527,15 @@
         <f t="shared" si="1"/>
         <v>122.08</v>
       </c>
-      <c r="H81" s="25" t="s">
+      <c r="H81" s="24" t="s">
         <v>237</v>
       </c>
     </row>
-    <row r="82" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A82" s="14" t="s">
         <v>62</v>
       </c>
-      <c r="B82" s="28" t="s">
+      <c r="B82" s="27" t="s">
         <v>238</v>
       </c>
       <c r="C82" s="18" t="s">
@@ -3520,15 +3551,15 @@
         <f t="shared" si="1"/>
         <v>382.26</v>
       </c>
-      <c r="H82" s="24" t="s">
+      <c r="H82" s="23" t="s">
         <v>238</v>
       </c>
     </row>
-    <row r="83" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A83" s="15" t="s">
         <v>63</v>
       </c>
-      <c r="B83" s="28" t="s">
+      <c r="B83" s="27" t="s">
         <v>239</v>
       </c>
       <c r="C83" s="19" t="s">
@@ -3544,15 +3575,15 @@
         <f t="shared" si="1"/>
         <v>95.56</v>
       </c>
-      <c r="H83" s="25" t="s">
+      <c r="H83" s="24" t="s">
         <v>239</v>
       </c>
     </row>
-    <row r="84" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A84" s="14" t="s">
         <v>64</v>
       </c>
-      <c r="B84" s="28" t="s">
+      <c r="B84" s="27" t="s">
         <v>240</v>
       </c>
       <c r="C84" s="18" t="s">
@@ -3568,15 +3599,15 @@
         <f t="shared" si="1"/>
         <v>49.95</v>
       </c>
-      <c r="H84" s="24" t="s">
+      <c r="H84" s="23" t="s">
         <v>240</v>
       </c>
     </row>
-    <row r="85" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A85" s="15" t="s">
         <v>35</v>
       </c>
-      <c r="B85" s="28" t="s">
+      <c r="B85" s="27" t="s">
         <v>241</v>
       </c>
       <c r="C85" s="19" t="s">
@@ -3592,15 +3623,15 @@
         <f t="shared" si="1"/>
         <v>6.02</v>
       </c>
-      <c r="H85" s="25" t="s">
+      <c r="H85" s="24" t="s">
         <v>241</v>
       </c>
     </row>
-    <row r="86" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A86" s="14" t="s">
         <v>63</v>
       </c>
-      <c r="B86" s="28" t="s">
+      <c r="B86" s="27" t="s">
         <v>242</v>
       </c>
       <c r="C86" s="18" t="s">
@@ -3616,15 +3647,15 @@
         <f t="shared" si="1"/>
         <v>2.3199999999999998</v>
       </c>
-      <c r="H86" s="24" t="s">
+      <c r="H86" s="23" t="s">
         <v>242</v>
       </c>
     </row>
-    <row r="87" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A87" s="15" t="s">
         <v>65</v>
       </c>
-      <c r="B87" s="28" t="s">
+      <c r="B87" s="27" t="s">
         <v>243</v>
       </c>
       <c r="C87" s="15" t="s">
@@ -3640,15 +3671,15 @@
         <f t="shared" si="1"/>
         <v>47.96</v>
       </c>
-      <c r="H87" s="25" t="s">
+      <c r="H87" s="24" t="s">
         <v>243</v>
       </c>
     </row>
-    <row r="88" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A88" s="14" t="s">
         <v>63</v>
       </c>
-      <c r="B88" s="28" t="s">
+      <c r="B88" s="27" t="s">
         <v>244</v>
       </c>
       <c r="C88" s="14" t="s">
@@ -3664,15 +3695,15 @@
         <f t="shared" si="1"/>
         <v>9.99</v>
       </c>
-      <c r="H88" s="24" t="s">
+      <c r="H88" s="23" t="s">
         <v>244</v>
       </c>
     </row>
-    <row r="89" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A89" s="15" t="s">
         <v>66</v>
       </c>
-      <c r="B89" s="28" t="s">
+      <c r="B89" s="27" t="s">
         <v>245</v>
       </c>
       <c r="C89" s="19" t="s">
@@ -3688,18 +3719,18 @@
         <f t="shared" si="1"/>
         <v>29.26</v>
       </c>
-      <c r="H89" s="25" t="s">
+      <c r="H89" s="24" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="90" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A90" s="14" t="s">
         <v>67</v>
       </c>
-      <c r="B90" s="28" t="s">
+      <c r="B90" s="27" t="s">
         <v>246</v>
       </c>
-      <c r="C90" s="23" t="s">
+      <c r="C90" s="22" t="s">
         <v>150</v>
       </c>
       <c r="D90" s="8">
@@ -3712,15 +3743,15 @@
         <f t="shared" si="1"/>
         <v>669.68</v>
       </c>
-      <c r="H90" s="24" t="s">
+      <c r="H90" s="23" t="s">
         <v>246</v>
       </c>
     </row>
-    <row r="91" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A91" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="B91" s="28" t="s">
+      <c r="B91" s="27" t="s">
         <v>247</v>
       </c>
       <c r="C91" s="19" t="s">
@@ -3736,15 +3767,15 @@
         <f t="shared" si="1"/>
         <v>12.61</v>
       </c>
-      <c r="H91" s="25" t="s">
+      <c r="H91" s="24" t="s">
         <v>247</v>
       </c>
     </row>
-    <row r="92" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A92" s="14" t="s">
         <v>68</v>
       </c>
-      <c r="B92" s="28"/>
+      <c r="B92" s="27"/>
       <c r="C92" s="14" t="s">
         <v>152</v>
       </c>
@@ -3758,15 +3789,15 @@
         <f t="shared" si="1"/>
         <v>20.9</v>
       </c>
-      <c r="H92" s="26" t="s">
+      <c r="H92" s="25" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="93" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A93" s="15" t="s">
         <v>68</v>
       </c>
-      <c r="B93" s="28"/>
+      <c r="B93" s="27"/>
       <c r="C93" s="15" t="s">
         <v>153</v>
       </c>
@@ -3780,15 +3811,15 @@
         <f t="shared" si="1"/>
         <v>6.5400000000000009</v>
       </c>
-      <c r="H93" s="27" t="s">
+      <c r="H93" s="26" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="94" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A94" s="14" t="s">
         <v>69</v>
       </c>
-      <c r="B94" s="28"/>
+      <c r="B94" s="27"/>
       <c r="C94" s="14">
         <v>156665159304</v>
       </c>
@@ -3802,15 +3833,15 @@
         <f t="shared" si="1"/>
         <v>107.91</v>
       </c>
-      <c r="H94" s="26" t="s">
+      <c r="H94" s="25" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="95" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A95" s="15" t="s">
         <v>67</v>
       </c>
-      <c r="B95" s="28" t="s">
+      <c r="B95" s="27" t="s">
         <v>246</v>
       </c>
       <c r="C95" s="15" t="s">
@@ -3826,15 +3857,15 @@
         <f t="shared" si="1"/>
         <v>502.26</v>
       </c>
-      <c r="H95" s="25" t="s">
+      <c r="H95" s="24" t="s">
         <v>246</v>
       </c>
     </row>
-    <row r="96" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A96" s="14" t="s">
         <v>70</v>
       </c>
-      <c r="B96" s="28" t="s">
+      <c r="B96" s="27" t="s">
         <v>258</v>
       </c>
       <c r="C96" s="14">
@@ -3850,15 +3881,15 @@
         <f t="shared" si="1"/>
         <v>405</v>
       </c>
-      <c r="H96" s="24" t="s">
+      <c r="H96" s="23" t="s">
         <v>248</v>
       </c>
     </row>
-    <row r="97" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A97" s="15" t="s">
         <v>66</v>
       </c>
-      <c r="B97" s="28" t="s">
+      <c r="B97" s="27" t="s">
         <v>259</v>
       </c>
       <c r="C97" s="12" t="s">
@@ -3874,15 +3905,15 @@
         <f t="shared" si="1"/>
         <v>37.4</v>
       </c>
-      <c r="H97" s="25" t="s">
+      <c r="H97" s="24" t="s">
         <v>249</v>
       </c>
     </row>
-    <row r="98" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A98" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="B98" s="28" t="s">
+      <c r="B98" s="27" t="s">
         <v>250</v>
       </c>
       <c r="C98" s="13" t="s">
@@ -3898,15 +3929,15 @@
         <f t="shared" si="1"/>
         <v>20.91</v>
       </c>
-      <c r="H98" s="24" t="s">
+      <c r="H98" s="23" t="s">
         <v>250</v>
       </c>
     </row>
-    <row r="99" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A99" s="15" t="s">
         <v>61</v>
       </c>
-      <c r="B99" s="28" t="s">
+      <c r="B99" s="27" t="s">
         <v>260</v>
       </c>
       <c r="C99" s="12" t="s">
@@ -3922,15 +3953,15 @@
         <f t="shared" si="1"/>
         <v>79.099999999999994</v>
       </c>
-      <c r="H99" s="25" t="s">
+      <c r="H99" s="24" t="s">
         <v>251</v>
       </c>
     </row>
-    <row r="100" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A100" s="14" t="s">
         <v>71</v>
       </c>
-      <c r="B100" s="28" t="s">
+      <c r="B100" s="27" t="s">
         <v>252</v>
       </c>
       <c r="C100" s="18" t="s">
@@ -3946,15 +3977,15 @@
         <f t="shared" si="1"/>
         <v>16.260000000000002</v>
       </c>
-      <c r="H100" s="24" t="s">
+      <c r="H100" s="23" t="s">
         <v>252</v>
       </c>
     </row>
-    <row r="101" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A101" s="15" t="s">
         <v>72</v>
       </c>
-      <c r="B101" s="28" t="s">
+      <c r="B101" s="27" t="s">
         <v>253</v>
       </c>
       <c r="C101" s="19" t="s">
@@ -3970,15 +4001,15 @@
         <f t="shared" si="1"/>
         <v>6.94</v>
       </c>
-      <c r="H101" s="25" t="s">
+      <c r="H101" s="24" t="s">
         <v>253</v>
       </c>
     </row>
-    <row r="102" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A102" s="14" t="s">
         <v>73</v>
       </c>
-      <c r="B102" s="28" t="s">
+      <c r="B102" s="27" t="s">
         <v>254</v>
       </c>
       <c r="C102" s="18" t="s">
@@ -3994,15 +4025,15 @@
         <f t="shared" si="1"/>
         <v>7.91</v>
       </c>
-      <c r="H102" s="24" t="s">
+      <c r="H102" s="23" t="s">
         <v>254</v>
       </c>
     </row>
-    <row r="103" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A103" s="15" t="s">
         <v>74</v>
       </c>
-      <c r="B103" s="28" t="s">
+      <c r="B103" s="27" t="s">
         <v>255</v>
       </c>
       <c r="C103" s="19" t="s">
@@ -4018,37 +4049,65 @@
         <f t="shared" si="1"/>
         <v>7.68</v>
       </c>
-      <c r="H103" s="25" t="s">
+      <c r="H103" s="24" t="s">
         <v>255</v>
       </c>
     </row>
-    <row r="104" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A104" s="22"/>
-      <c r="B104" s="22"/>
-      <c r="C104" s="22"/>
-      <c r="H104" s="11"/>
-    </row>
-    <row r="105" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A105" s="22"/>
-      <c r="B105" s="22"/>
-      <c r="C105" s="22"/>
-      <c r="H105" s="11"/>
-    </row>
-    <row r="106" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A106" s="22"/>
-      <c r="B106" s="22"/>
-      <c r="C106" s="22"/>
+    <row r="104" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A104" s="28" t="s">
+        <v>74</v>
+      </c>
+      <c r="B104" s="29" t="s">
+        <v>261</v>
+      </c>
+      <c r="C104" s="30"/>
+      <c r="D104" s="31"/>
+      <c r="E104" s="31"/>
+      <c r="F104" s="32">
+        <f>D104*E104</f>
+        <v>0</v>
+      </c>
+      <c r="G104" s="33"/>
+      <c r="H104" s="34"/>
+      <c r="I104" s="33"/>
+      <c r="J104" s="33"/>
+      <c r="K104" s="33"/>
+    </row>
+    <row r="105" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A105" s="28" t="s">
+        <v>72</v>
+      </c>
+      <c r="B105" s="29" t="s">
+        <v>262</v>
+      </c>
+      <c r="C105" s="30"/>
+      <c r="D105" s="31"/>
+      <c r="E105" s="31"/>
+      <c r="F105" s="32">
+        <f>D105*E105</f>
+        <v>0</v>
+      </c>
+      <c r="G105" s="33"/>
+      <c r="H105" s="34"/>
+      <c r="I105" s="33"/>
+      <c r="J105" s="33"/>
+      <c r="K105" s="33"/>
+    </row>
+    <row r="106" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A106" s="11"/>
+      <c r="B106" s="11"/>
+      <c r="C106" s="11"/>
       <c r="H106" s="11"/>
     </row>
-    <row r="107" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A107" s="22"/>
-      <c r="B107" s="22"/>
-      <c r="C107" s="22"/>
+    <row r="107" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A107" s="11"/>
+      <c r="B107" s="11"/>
+      <c r="C107" s="11"/>
       <c r="H107" s="11"/>
     </row>
-    <row r="109" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:11" x14ac:dyDescent="0.2">
       <c r="F109" s="6">
-        <f>SUM(F2:F103)</f>
+        <f>SUM(F2:F105)</f>
         <v>9533.0300000000043</v>
       </c>
     </row>

</xml_diff>